<commit_message>
Save library recording testcomplete - 615212be-c784-415a-ae45-d72b494a9f6f - 2026-10-12T09:26:13.954472Z
</commit_message>
<xml_diff>
--- a/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/615212be-c784-415a-ae45-d72b494a9f6f/resources/azure-devops.xlsx
+++ b/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/615212be-c784-415a-ae45-d72b494a9f6f/resources/azure-devops.xlsx
@@ -495,7 +495,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)", "x": 123, "y": 322, "tag": "input", "schema_version": 1, "strict": true}</t>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)", "schema_version": 1, "strict": true, "tag": "input", "x": 123, "y": 322}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -547,7 +547,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)", "x": 115, "y": 416, "tag": "input", "schema_version": 1, "strict": true}</t>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)", "schema_version": 1, "strict": true, "tag": "input", "x": 115, "y": 416}</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>

</xml_diff>